<commit_message>
changed and fixed the sql ted the sql tables to be exactly the same as the client request which is shown in the csv file i pushed last
</commit_message>
<xml_diff>
--- a/docs/Data.xlsx
+++ b/docs/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/de348250dbb8bac6/Desktop/Temporary/02340311 - Yearly Project in Software Eng.-Stage a/GhostHouses/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE575DA1-A216-4327-97FD-75683317FA35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{EE575DA1-A216-4327-97FD-75683317FA35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68274AFB-7E72-4176-8EBD-B0729CF033A9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{33D2E388-C745-428F-9501-C6EDF39C853A}"/>
   </bookViews>
@@ -83,9 +83,6 @@
     <t>BldName</t>
   </si>
   <si>
-    <t>BIdSivug</t>
-  </si>
-  <si>
     <t>סיווג</t>
   </si>
   <si>
@@ -570,6 +567,9 @@
   </si>
   <si>
     <t>פיקוח על הבניה</t>
+  </si>
+  <si>
+    <t>BldSivug</t>
   </si>
 </sst>
 </file>
@@ -724,7 +724,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -756,16 +756,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -786,25 +783,6 @@
   </cellStyles>
   <dxfs count="11">
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -946,13 +924,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -970,6 +941,32 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -985,15 +982,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9C5488EF-EF21-41E0-93DC-CA9EDB1B8BBE}" name="Table1" displayName="Table1" ref="A1:F71" totalsRowShown="0" headerRowDxfId="0" dataDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9C5488EF-EF21-41E0-93DC-CA9EDB1B8BBE}" name="Table1" displayName="Table1" ref="A1:F71" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
   <autoFilter ref="A1:F71" xr:uid="{9C5488EF-EF21-41E0-93DC-CA9EDB1B8BBE}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{1D85ABA0-863B-42A9-A006-27BE12567AFC}" name="Category" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{13AF838B-70AE-422F-AB9C-20A9B9A73582}" name="Field ID" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{2D8D6BE4-0556-40C4-8F5F-CA22B2E7385B}" name="Field Name" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{31F07A81-7037-47EB-85FC-7AB8E0AD9886}" name="Type" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{95163747-2F5F-454D-B645-44A51D632F47}" name="Foreign Field ID" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{254D2933-47DD-4BA1-A77F-AF0E6BCF13CC}" name="Include in event log (date of change &amp; the change)" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{1D85ABA0-863B-42A9-A006-27BE12567AFC}" name="Category" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{13AF838B-70AE-422F-AB9C-20A9B9A73582}" name="Field ID" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{2D8D6BE4-0556-40C4-8F5F-CA22B2E7385B}" name="Field Name" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{31F07A81-7037-47EB-85FC-7AB8E0AD9886}" name="Type" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{95163747-2F5F-454D-B645-44A51D632F47}" name="Foreign Field ID" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{254D2933-47DD-4BA1-A77F-AF0E6BCF13CC}" name="Include in event log (date of change &amp; the change)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1316,7 +1313,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C406DF-314D-4084-8AC5-45D6280A6294}">
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.5546875" style="7" bestFit="1" customWidth="1"/>
@@ -1349,23 +1346,23 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="9"/>
-      <c r="F2" s="16"/>
+      <c r="F2" s="15"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="9" t="s">
@@ -1378,10 +1375,10 @@
         <v>11</v>
       </c>
       <c r="E3" s="9"/>
-      <c r="F3" s="16"/>
+      <c r="F3" s="15"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -1394,1260 +1391,1237 @@
         <v>11</v>
       </c>
       <c r="E4" s="9"/>
-      <c r="F4" s="16"/>
+      <c r="F4" s="15"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="9"/>
-      <c r="F5" s="16"/>
+      <c r="F5" s="15"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="D6" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="9" t="s">
+      <c r="F6" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="15" t="s">
+      <c r="C7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="9" t="s">
+      <c r="B8" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="9" t="s">
+      <c r="C8" s="9" t="s">
         <v>21</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>22</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="9"/>
-      <c r="F8" s="16" t="s">
-        <v>64</v>
+      <c r="F8" s="15" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="D9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="E9" s="9"/>
+      <c r="F9" s="15"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="16"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="9" t="s">
+      <c r="C10" s="9" t="s">
         <v>26</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>27</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="9"/>
-      <c r="F10" s="16" t="s">
-        <v>64</v>
+      <c r="F10" s="15" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="C11" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="E11" s="9"/>
+      <c r="F11" s="15"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="16"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="9" t="s">
+      <c r="C12" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="9"/>
+      <c r="F12" s="15"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="16"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="9" t="s">
+      <c r="C13" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="9"/>
+      <c r="F13" s="15"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="16"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="9" t="s">
+      <c r="C14" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="9"/>
+      <c r="F14" s="15"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="16"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="9" t="s">
+      <c r="C15" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="9"/>
+      <c r="F15" s="15"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="16"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16" s="9" t="s">
+      <c r="C16" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="9"/>
+      <c r="F16" s="15"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="9"/>
-      <c r="F16" s="16"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>36</v>
-      </c>
       <c r="C17" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="9"/>
-      <c r="F17" s="16"/>
+      <c r="F17" s="15"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="15" t="s">
-        <v>28</v>
+      <c r="A18" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="B18" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="D18" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="9"/>
+      <c r="F18" s="15"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18" s="9"/>
-      <c r="F18" s="16"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="9" t="s">
+      <c r="C19" s="9" t="s">
         <v>39</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>40</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E19" s="9"/>
-      <c r="F19" s="16"/>
+      <c r="F19" s="15"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="15" t="s">
-        <v>28</v>
+      <c r="A20" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="B20" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>41</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>42</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E20" s="9"/>
-      <c r="F20" s="16"/>
+      <c r="F20" s="15"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="15" t="s">
-        <v>28</v>
+      <c r="A21" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="B21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="D21" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="9"/>
+      <c r="F21" s="15"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E21" s="9"/>
-      <c r="F21" s="16"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="9" t="s">
+      <c r="C22" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22" s="9" t="s">
+      <c r="F22" s="15"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F22" s="16"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="9" t="s">
+      <c r="C23" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E23" s="9" t="s">
+      <c r="F23" s="15"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="F23" s="16"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B24" s="9" t="s">
+      <c r="C24" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E24" s="9"/>
+      <c r="F24" s="15"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E24" s="9"/>
-      <c r="F24" s="16"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B25" s="9" t="s">
+      <c r="C25" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25" s="9"/>
+      <c r="F25" s="15"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E25" s="9"/>
-      <c r="F25" s="16"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>51</v>
-      </c>
       <c r="C26" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D26" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E26" s="9"/>
-      <c r="F26" s="16" t="s">
-        <v>64</v>
+      <c r="F26" s="15" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="15" t="s">
-        <v>28</v>
+      <c r="A27" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="B27" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>52</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>53</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E27" s="9"/>
-      <c r="F27" s="16" t="s">
-        <v>64</v>
+      <c r="F27" s="15" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="15" t="s">
-        <v>28</v>
+      <c r="A28" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="B28" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="9"/>
+      <c r="F28" s="15"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E28" s="9"/>
-      <c r="F28" s="16"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="15" t="s">
+      <c r="B29" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="C29" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="D29" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F29" s="15"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="D29" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E29" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F29" s="16"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>58</v>
-      </c>
       <c r="C30" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E30" s="9"/>
-      <c r="F30" s="16"/>
+      <c r="F30" s="15"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="15" t="s">
-        <v>55</v>
+      <c r="A31" s="14" t="s">
+        <v>54</v>
       </c>
       <c r="B31" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" s="9" t="s">
         <v>59</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>60</v>
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F31" s="16"/>
+        <v>47</v>
+      </c>
+      <c r="F31" s="15"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="15" t="s">
-        <v>55</v>
+      <c r="A32" s="14" t="s">
+        <v>54</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E32" s="9"/>
-      <c r="F32" s="16"/>
+      <c r="F32" s="15"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="17" t="s">
-        <v>55</v>
+      <c r="A33" s="16" t="s">
+        <v>54</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E33" s="8"/>
-      <c r="F33" s="18" t="s">
-        <v>64</v>
+      <c r="F33" s="17" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="17" t="s">
-        <v>135</v>
+      <c r="A34" s="16" t="s">
+        <v>134</v>
       </c>
       <c r="B34" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E34" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C34" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E34" s="8" t="s">
+      <c r="F34" s="17"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B35" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="F34" s="18"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="B35" s="8" t="s">
+      <c r="C35" s="8" t="s">
         <v>83</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>84</v>
       </c>
       <c r="D35" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E35" s="8"/>
-      <c r="F35" s="18"/>
+      <c r="F35" s="17"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="17" t="s">
-        <v>135</v>
+      <c r="A36" s="16" t="s">
+        <v>134</v>
       </c>
       <c r="B36" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F36" s="17"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B37" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C37" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="D36" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="F36" s="18"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="B37" s="8" t="s">
+      <c r="D37" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="F37" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="C39" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="D37" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="F37" s="18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="C38" s="8" t="s">
+      <c r="D39" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B40" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D38" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="F38" s="18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C39" s="8" t="s">
+      <c r="C40" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F40" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C41" s="8" t="s">
         <v>142</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F39" s="18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C40" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="F40" s="18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>143</v>
       </c>
       <c r="D41" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E41" s="8"/>
-      <c r="F41" s="18"/>
+      <c r="F41" s="17"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="17" t="s">
-        <v>135</v>
+      <c r="A42" s="16" t="s">
+        <v>134</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D42" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E42" s="8"/>
-      <c r="F42" s="18"/>
+      <c r="F42" s="17"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="17" t="s">
-        <v>135</v>
+      <c r="A43" s="16" t="s">
+        <v>134</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D43" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E43" s="9"/>
-      <c r="F43" s="16"/>
+      <c r="F43" s="15"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="17" t="s">
+      <c r="A44" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" s="9"/>
+      <c r="F44" s="15"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F45" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="B44" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" s="9"/>
-      <c r="F44" s="16"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="17" t="s">
+      <c r="B46" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F46" s="15"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="B45" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E45" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="F45" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="C46" s="9" t="s">
+      <c r="B47" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C47" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="D46" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E46" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="F46" s="16"/>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="B47" s="9" t="s">
+      <c r="D47" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F47" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B48" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C48" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D47" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E47" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F47" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="B48" s="9" t="s">
+      <c r="D48" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F48" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B49" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="C48" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E48" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F48" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="B49" s="9" t="s">
+      <c r="C49" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="D49" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="D49" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E49" s="9" t="s">
+      <c r="F49" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B50" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="F49" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="B50" s="9" t="s">
+      <c r="C50" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="D50" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E50" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="D50" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E50" s="9" t="s">
+      <c r="F50" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B51" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="F50" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="B51" s="9" t="s">
+      <c r="C51" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="D51" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F51" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B52" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="D51" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E51" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F51" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="B52" s="9" t="s">
+      <c r="C52" s="9" t="s">
         <v>112</v>
-      </c>
-      <c r="C52" s="9" t="s">
-        <v>113</v>
       </c>
       <c r="D52" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E52" s="9"/>
-      <c r="F52" s="16" t="s">
-        <v>64</v>
+      <c r="F52" s="15" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="15" t="s">
-        <v>136</v>
+      <c r="A53" s="14" t="s">
+        <v>135</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D53" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E53" s="9"/>
-      <c r="F53" s="16" t="s">
-        <v>64</v>
+      <c r="F53" s="15" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="15" t="s">
-        <v>136</v>
+      <c r="A54" s="14" t="s">
+        <v>135</v>
       </c>
       <c r="B54" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C54" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="D54" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54" s="9"/>
+      <c r="F54" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B55" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="D54" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E54" s="9"/>
-      <c r="F54" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="B55" s="9" t="s">
+      <c r="C55" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="D55" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F55" s="15"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="D55" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E55" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F55" s="16"/>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="15" t="s">
+      <c r="B56" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="B56" s="9" t="s">
+      <c r="C56" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E56" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F56" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B57" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="C56" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="D56" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E56" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F56" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="B57" s="9" t="s">
+      <c r="C57" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="D57" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F57" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B58" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="D57" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E57" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F57" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="B58" s="9" t="s">
+      <c r="C58" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="D58" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F58" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B59" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="D58" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E58" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F58" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="B59" s="9" t="s">
+      <c r="C59" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="D59" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D59" s="9" t="s">
+      <c r="E59" s="9"/>
+      <c r="F59" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="E59" s="9"/>
-      <c r="F59" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="15" t="s">
+      <c r="B60" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="B60" s="9" t="s">
+      <c r="C60" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="D60" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="D60" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E60" s="9" t="s">
+      <c r="F60" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="B61" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="F60" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="B61" s="9" t="s">
+      <c r="C61" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="D61" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="D61" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E61" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="F61" s="16" t="s">
-        <v>64</v>
+      <c r="F61" s="15" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="17" t="s">
-        <v>128</v>
+      <c r="A62" s="16" t="s">
+        <v>127</v>
       </c>
       <c r="B62" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="C62" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="C62" s="8" t="s">
+      <c r="D62" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E62" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="D62" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E62" s="8" t="s">
+      <c r="F62" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="F62" s="18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="17" t="s">
+      <c r="B63" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="B63" s="8" t="s">
+      <c r="C63" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="C63" s="8" t="s">
+      <c r="D63" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E63" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="D63" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E63" s="8" t="s">
+      <c r="F63" s="17"/>
+    </row>
+    <row r="64" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A64" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="B64" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="F63" s="18"/>
-    </row>
-    <row r="64" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A64" s="17" t="s">
-        <v>155</v>
-      </c>
-      <c r="B64" s="8" t="s">
+      <c r="C64" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="D64" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="F64" s="17"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="B65" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="C64" s="8" t="s">
+      <c r="C65" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="D64" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E64" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="F64" s="18"/>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A65" s="17" t="s">
-        <v>155</v>
-      </c>
-      <c r="B65" s="8" t="s">
+      <c r="D65" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="C65" s="8" t="s">
+      <c r="F65" s="17"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C66" s="8" t="s">
         <v>175</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E65" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="F65" s="18"/>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A66" s="17" t="s">
-        <v>155</v>
-      </c>
-      <c r="B66" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="C66" s="8" t="s">
-        <v>176</v>
       </c>
       <c r="D66" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E66" s="8"/>
-      <c r="F66" s="18"/>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A67" s="17" t="s">
-        <v>155</v>
+      <c r="F66" s="17"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="16" t="s">
+        <v>154</v>
       </c>
       <c r="B67" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C67" s="8" t="s">
         <v>163</v>
-      </c>
-      <c r="C67" s="8" t="s">
-        <v>164</v>
       </c>
       <c r="D67" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E67" s="8"/>
-      <c r="F67" s="18"/>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A68" s="17" t="s">
+      <c r="F67" s="17"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="B68" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="B68" s="8" t="s">
+      <c r="C68" s="8" t="s">
         <v>166</v>
-      </c>
-      <c r="C68" s="8" t="s">
-        <v>167</v>
       </c>
       <c r="D68" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E68" s="8"/>
-      <c r="F68" s="18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A69" s="17" t="s">
-        <v>165</v>
+      <c r="F68" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="16" t="s">
+        <v>164</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D69" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E69" s="8"/>
-      <c r="F69" s="18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A70" s="15" t="s">
-        <v>165</v>
+      <c r="F69" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="14" t="s">
+        <v>164</v>
       </c>
       <c r="B70" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="C70" s="9" t="s">
         <v>169</v>
-      </c>
-      <c r="C70" s="9" t="s">
-        <v>170</v>
       </c>
       <c r="D70" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E70" s="9"/>
-      <c r="F70" s="16" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F70" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E71" s="2"/>
       <c r="F71" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="11"/>
       <c r="B72" s="11"/>
       <c r="C72" s="11"/>
       <c r="D72" s="11"/>
       <c r="E72" s="11"/>
       <c r="F72" s="11"/>
-      <c r="G72" s="12"/>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A73" s="13"/>
-      <c r="B73" s="13"/>
-      <c r="C73" s="13"/>
-      <c r="D73" s="13"/>
-      <c r="E73" s="13"/>
-      <c r="F73" s="13"/>
-      <c r="G73" s="12"/>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A74" s="14"/>
-      <c r="B74" s="14"/>
-      <c r="C74" s="14"/>
-      <c r="D74" s="14"/>
-      <c r="E74" s="14"/>
-      <c r="F74" s="14"/>
-      <c r="G74" s="12"/>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A75" s="13"/>
-      <c r="B75" s="13"/>
-      <c r="C75" s="13"/>
-      <c r="D75" s="13"/>
-      <c r="E75" s="13"/>
-      <c r="F75" s="13"/>
-      <c r="G75" s="12"/>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A76" s="14"/>
-      <c r="B76" s="14"/>
-      <c r="C76" s="14"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="14"/>
-      <c r="F76" s="14"/>
-      <c r="G76" s="12"/>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A77" s="12"/>
-      <c r="B77" s="12"/>
-      <c r="C77" s="12"/>
-      <c r="D77" s="12"/>
-      <c r="E77" s="12"/>
-      <c r="F77" s="12"/>
-      <c r="G77" s="12"/>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A78" s="12"/>
-      <c r="B78" s="12"/>
-      <c r="C78" s="12"/>
-      <c r="D78" s="12"/>
-      <c r="E78" s="12"/>
-      <c r="F78" s="12"/>
-      <c r="G78" s="12"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="12"/>
+      <c r="B73" s="12"/>
+      <c r="C73" s="12"/>
+      <c r="D73" s="12"/>
+      <c r="E73" s="12"/>
+      <c r="F73" s="12"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" s="13"/>
+      <c r="B74" s="13"/>
+      <c r="C74" s="13"/>
+      <c r="D74" s="13"/>
+      <c r="E74" s="13"/>
+      <c r="F74" s="13"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" s="12"/>
+      <c r="B75" s="12"/>
+      <c r="C75" s="12"/>
+      <c r="D75" s="12"/>
+      <c r="E75" s="12"/>
+      <c r="F75" s="12"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" s="13"/>
+      <c r="B76" s="13"/>
+      <c r="C76" s="13"/>
+      <c r="D76" s="13"/>
+      <c r="E76" s="13"/>
+      <c r="F76" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>